<commit_message>
fix: the key inventory holds the labels the manifest now uses
Commits 2dbcded and 9aeacd9 changed the navigation and tab labels to the
keys todo, todo-list and predefined-todo-list, but the inventory still
held to-do. Five tests in translation-inventory.test.js failed on main.
The inventory and its workbook now hold the three keys, and the README
says what the labels are and what the panel's page gate still does
with them.
</commit_message>
<xml_diff>
--- a/frontend/translations/todo-translation-keys.xlsx
+++ b/frontend/translations/todo-translation-keys.xlsx
@@ -66,229 +66,243 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">to-do</t>
+          <t xml:space="preserve">predefined-todo-list</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.add</t>
+          <t xml:space="preserve">todo</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.add-computer-todo-title</t>
+          <t xml:space="preserve">todo-list</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.add-computer-todo-tooltip</t>
+          <t xml:space="preserve">todo.add</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.add-list</t>
+          <t xml:space="preserve">todo.add-computer-todo-title</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.add-todo</t>
+          <t xml:space="preserve">todo.add-computer-todo-tooltip</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.cancel</t>
+          <t xml:space="preserve">todo.add-list</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.computer</t>
+          <t xml:space="preserve">todo.add-todo</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.computer-todo-added</t>
+          <t xml:space="preserve">todo.cancel</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.delete</t>
+          <t xml:space="preserve">todo.computer</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.edit</t>
+          <t xml:space="preserve">todo.computer-todo-added</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-no-access</t>
+          <t xml:space="preserve">todo.delete</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-read-only</t>
+          <t xml:space="preserve">todo.edit</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-reference</t>
+          <t xml:space="preserve">todo.error-no-access</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-request-failed</t>
+          <t xml:space="preserve">todo.error-read-only</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-session-ended</t>
+          <t xml:space="preserve">todo.error-reference</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.error-unavailable</t>
+          <t xml:space="preserve">todo.error-request-failed</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-placeholder</t>
+          <t xml:space="preserve">todo.error-session-ended</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-required</t>
+          <t xml:space="preserve">todo.error-unavailable</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-placeholder</t>
+          <t xml:space="preserve">todo.list-items-placeholder</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-required</t>
+          <t xml:space="preserve">todo.list-items-required</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-name-placeholder</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-name-required</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer</t>
+          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer-todos</t>
+          <t xml:space="preserve">todo.new-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-predefined-lists</t>
+          <t xml:space="preserve">todo.no-computer</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-todos</t>
+          <t xml:space="preserve">todo.no-computer-todos</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.predefined-title</t>
+          <t xml:space="preserve">todo.no-predefined-lists</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only</t>
+          <t xml:space="preserve">todo.no-todos</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only-suffix</t>
+          <t xml:space="preserve">todo.predefined-title</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.save</t>
+          <t xml:space="preserve">todo.read-only</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.signed-in-as</t>
+          <t xml:space="preserve">todo.read-only-suffix</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.save</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.signed-in-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">todo.title</t>
         </is>

</xml_diff>

<commit_message>
fix: the Predefined page's label is its sub tab, todo-predefined
The panel opens a page only for a user holding the tab named like its label,
and Core names this page's sub tab todo-predefined, so predefined-todo-list
hid the page from everyone and failed forge validate. The inventory and the
workbook carry the new key, and the open inventory test is now a real one.
</commit_message>
<xml_diff>
--- a/frontend/translations/todo-translation-keys.xlsx
+++ b/frontend/translations/todo-translation-keys.xlsx
@@ -66,21 +66,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">predefined-todo-list</t>
+          <t xml:space="preserve">todo</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo</t>
+          <t xml:space="preserve">todo-list</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo-list</t>
+          <t xml:space="preserve">todo-predefined</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update todo plugin backend and frontend-harb changes
</commit_message>
<xml_diff>
--- a/frontend/translations/todo-translation-keys.xlsx
+++ b/frontend/translations/todo-translation-keys.xlsx
@@ -185,110 +185,131 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-placeholder</t>
+          <t xml:space="preserve">todo.export</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-required</t>
+          <t xml:space="preserve">todo.export-failed</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-placeholder</t>
+          <t xml:space="preserve">todo.exporting</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-required</t>
+          <t xml:space="preserve">todo.list-items-placeholder</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-items-required</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-name-placeholder</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer</t>
+          <t xml:space="preserve">todo.list-name-required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer-todos</t>
+          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-predefined-lists</t>
+          <t xml:space="preserve">todo.new-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-todos</t>
+          <t xml:space="preserve">todo.no-computer</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.predefined-title</t>
+          <t xml:space="preserve">todo.no-computer-todos</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only</t>
+          <t xml:space="preserve">todo.no-predefined-lists</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only-suffix</t>
+          <t xml:space="preserve">todo.no-todos</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.save</t>
+          <t xml:space="preserve">todo.predefined-title</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.signed-in-as</t>
+          <t xml:space="preserve">todo.read-only</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.read-only-suffix</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.save</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.signed-in-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t xml:space="preserve">todo.title</t>
         </is>

</xml_diff>

<commit_message>
feat: add Todo user and system settings sections to manifest and implement corresponding modules
- Introduced new settings sections for user and system in manifest.json and pulsar.yaml.
- Created TodoUserSettings and TodoSystemSettings modules to handle user-specific and system-specific settings.
- Updated tests to cover the new settings sections and their functionalities.
- Enhanced translation keys for better localization support.
</commit_message>
<xml_diff>
--- a/frontend/translations/todo-translation-keys.xlsx
+++ b/frontend/translations/todo-translation-keys.xlsx
@@ -199,110 +199,145 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-placeholder</t>
+          <t xml:space="preserve">todo.export</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-items-required</t>
+          <t xml:space="preserve">todo.export-failed</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-placeholder</t>
+          <t xml:space="preserve">todo.exporting</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.list-name-required</t>
+          <t xml:space="preserve">todo.list-items-placeholder</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-items-required</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.new-todo-placeholder</t>
+          <t xml:space="preserve">todo.list-name-placeholder</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer</t>
+          <t xml:space="preserve">todo.list-name-required</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-computer-todos</t>
+          <t xml:space="preserve">todo.new-computer-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-predefined-lists</t>
+          <t xml:space="preserve">todo.new-todo-placeholder</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.no-todos</t>
+          <t xml:space="preserve">todo.no-computer</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.predefined-title</t>
+          <t xml:space="preserve">todo.no-computer-todos</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only</t>
+          <t xml:space="preserve">todo.no-predefined-lists</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.read-only-suffix</t>
+          <t xml:space="preserve">todo.no-todos</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.save</t>
+          <t xml:space="preserve">todo.open-todos</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">todo.signed-in-as</t>
+          <t xml:space="preserve">todo.predefined-title</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.read-only</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.read-only-suffix</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.save</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.service-status</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">todo.signed-in-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t xml:space="preserve">todo.title</t>
         </is>

</xml_diff>